<commit_message>
fix(pa): preserve catalog fields and add programmer review submission
</commit_message>
<xml_diff>
--- a/esap/programacion/resultados/2026-1/catalogo-importable-2026-1.xlsx
+++ b/esap/programacion/resultados/2026-1/catalogo-importable-2026-1.xlsx
@@ -497,10 +497,10 @@
         <v>TRUE</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>pregrado_sede_central</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>Pregrado Sede Central (AP/EP) - Bloque Fijo</v>
       </c>
       <c r="N2" t="str">
         <v/>
@@ -544,10 +544,10 @@
         <v>TRUE</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>pregrado_sede_central</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>Pregrado Sede Central (AP/EP) - Bloque Fijo</v>
       </c>
       <c r="N3" t="str">
         <v/>
@@ -591,10 +591,10 @@
         <v>TRUE</v>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>pregrado_territorial</v>
       </c>
       <c r="M4" t="str">
-        <v/>
+        <v>APT / Territorial - 16h por credito</v>
       </c>
       <c r="N4" t="str">
         <v/>
@@ -638,10 +638,10 @@
         <v>TRUE</v>
       </c>
       <c r="L5" t="str">
-        <v/>
+        <v>pregrado_sede_central</v>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>Pregrado Sede Central (AP/EP) - Bloque Fijo</v>
       </c>
       <c r="N5" t="str">
         <v/>
@@ -685,10 +685,10 @@
         <v>TRUE</v>
       </c>
       <c r="L6" t="str">
-        <v/>
+        <v>especializacion</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>Especializacion - 16h por credito</v>
       </c>
       <c r="N6" t="str">
         <v/>
@@ -732,10 +732,10 @@
         <v>TRUE</v>
       </c>
       <c r="L7" t="str">
-        <v/>
+        <v>especializacion</v>
       </c>
       <c r="M7" t="str">
-        <v/>
+        <v>Especializacion - 16h por credito</v>
       </c>
       <c r="N7" t="str">
         <v/>
@@ -779,10 +779,10 @@
         <v>TRUE</v>
       </c>
       <c r="L8" t="str">
-        <v/>
+        <v>especializacion</v>
       </c>
       <c r="M8" t="str">
-        <v/>
+        <v>Especializacion - 16h por credito</v>
       </c>
       <c r="N8" t="str">
         <v/>
@@ -826,10 +826,10 @@
         <v>TRUE</v>
       </c>
       <c r="L9" t="str">
-        <v/>
+        <v>especializacion</v>
       </c>
       <c r="M9" t="str">
-        <v/>
+        <v>Especializacion - 16h por credito</v>
       </c>
       <c r="N9" t="str">
         <v/>
@@ -873,10 +873,10 @@
         <v>TRUE</v>
       </c>
       <c r="L10" t="str">
-        <v/>
+        <v>especializacion</v>
       </c>
       <c r="M10" t="str">
-        <v/>
+        <v>Especializacion - 16h por credito</v>
       </c>
       <c r="N10" t="str">
         <v/>
@@ -920,10 +920,10 @@
         <v>TRUE</v>
       </c>
       <c r="L11" t="str">
-        <v/>
+        <v>especializacion</v>
       </c>
       <c r="M11" t="str">
-        <v/>
+        <v>Especializacion - 16h por credito</v>
       </c>
       <c r="N11" t="str">
         <v/>
@@ -967,10 +967,10 @@
         <v>TRUE</v>
       </c>
       <c r="L12" t="str">
-        <v/>
+        <v>especializacion</v>
       </c>
       <c r="M12" t="str">
-        <v/>
+        <v>Especializacion - 16h por credito</v>
       </c>
       <c r="N12" t="str">
         <v/>
@@ -1014,10 +1014,10 @@
         <v>TRUE</v>
       </c>
       <c r="L13" t="str">
-        <v/>
+        <v>maestria</v>
       </c>
       <c r="M13" t="str">
-        <v/>
+        <v>Maestria - 12h por credito</v>
       </c>
       <c r="N13" t="str">
         <v/>
@@ -1061,10 +1061,10 @@
         <v>TRUE</v>
       </c>
       <c r="L14" t="str">
-        <v/>
+        <v>maestria</v>
       </c>
       <c r="M14" t="str">
-        <v/>
+        <v>Maestria - 12h por credito</v>
       </c>
       <c r="N14" t="str">
         <v/>
@@ -1108,10 +1108,10 @@
         <v>TRUE</v>
       </c>
       <c r="L15" t="str">
-        <v/>
+        <v>maestria</v>
       </c>
       <c r="M15" t="str">
-        <v/>
+        <v>Maestria - 12h por credito</v>
       </c>
       <c r="N15" t="str">
         <v/>
@@ -1239,6 +1239,9 @@
       <c r="Q2" t="str">
         <v>NT-001</v>
       </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1346,7 +1349,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q4" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="R4" t="str">
         <v>AF-04</v>
@@ -1402,7 +1405,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q5" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="R5" t="str">
         <v>AF-04</v>
@@ -1740,6 +1743,9 @@
       <c r="Q11" t="str">
         <v>NT-003</v>
       </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1793,6 +1799,9 @@
       <c r="Q12" t="str">
         <v>NT-003</v>
       </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1846,6 +1855,9 @@
       <c r="Q13" t="str">
         <v>NT-004</v>
       </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -3019,6 +3031,9 @@
       <c r="Q34" t="str">
         <v>NT-003</v>
       </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -3072,6 +3087,9 @@
       <c r="Q35" t="str">
         <v>NT-003</v>
       </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -3123,7 +3141,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q36" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="R36" t="str">
         <v>AF-04</v>
@@ -3179,7 +3197,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q37" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="R37" t="str">
         <v>AF-04</v>
@@ -3741,6 +3759,9 @@
       <c r="Q47" t="str">
         <v>NT-002</v>
       </c>
+      <c r="R47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -4074,6 +4095,9 @@
       <c r="Q53" t="str">
         <v>NT-002</v>
       </c>
+      <c r="R53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -4239,6 +4263,9 @@
       <c r="Q56" t="str">
         <v>NT-003</v>
       </c>
+      <c r="R56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -4292,6 +4319,9 @@
       <c r="Q57" t="str">
         <v>NT-003</v>
       </c>
+      <c r="R57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -4345,6 +4375,9 @@
       <c r="Q58" t="str">
         <v>NT-002</v>
       </c>
+      <c r="R58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -4396,7 +4429,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q59" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="R59" t="str">
         <v>AF-04</v>
@@ -4676,7 +4709,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q64" t="str">
-        <v/>
+        <v>NT-034</v>
       </c>
       <c r="R64" t="str">
         <v>AF-04</v>
@@ -4734,6 +4767,9 @@
       <c r="Q65" t="str">
         <v>NT-001</v>
       </c>
+      <c r="R65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -4787,6 +4823,9 @@
       <c r="Q66" t="str">
         <v>NT-001</v>
       </c>
+      <c r="R66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -4896,6 +4935,9 @@
       <c r="Q68" t="str">
         <v>NT-001</v>
       </c>
+      <c r="R68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -5173,6 +5215,9 @@
       <c r="Q73" t="str">
         <v>NT-002</v>
       </c>
+      <c r="R73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -5338,6 +5383,9 @@
       <c r="Q76" t="str">
         <v>NT-003</v>
       </c>
+      <c r="R76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -5391,6 +5439,9 @@
       <c r="Q77" t="str">
         <v>NT-003</v>
       </c>
+      <c r="R77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -5500,6 +5551,9 @@
       <c r="Q79" t="str">
         <v>NT-007</v>
       </c>
+      <c r="R79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -5553,6 +5607,9 @@
       <c r="Q80" t="str">
         <v>NT-008</v>
       </c>
+      <c r="R80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -5886,6 +5943,9 @@
       <c r="Q86" t="str">
         <v>NT-009</v>
       </c>
+      <c r="R86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -6107,6 +6167,9 @@
       <c r="Q90" t="str">
         <v>NT-008</v>
       </c>
+      <c r="R90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -6328,6 +6391,9 @@
       <c r="Q94" t="str">
         <v>NT-002</v>
       </c>
+      <c r="R94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -6885,6 +6951,9 @@
       <c r="Q104" t="str">
         <v>NT-006</v>
       </c>
+      <c r="R104" t="str">
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -6994,6 +7063,9 @@
       <c r="Q106" t="str">
         <v>NT-009</v>
       </c>
+      <c r="R106" t="str">
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -7103,6 +7175,9 @@
       <c r="Q108" t="str">
         <v>NT-008</v>
       </c>
+      <c r="R108" t="str">
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -7156,6 +7231,9 @@
       <c r="Q109" t="str">
         <v>NT-005</v>
       </c>
+      <c r="R109" t="str">
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -7265,6 +7343,9 @@
       <c r="Q111" t="str">
         <v>NT-007</v>
       </c>
+      <c r="R111" t="str">
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -7430,6 +7511,9 @@
       <c r="Q114" t="str">
         <v>NT-008</v>
       </c>
+      <c r="R114" t="str">
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -7819,6 +7903,9 @@
       <c r="Q121" t="str">
         <v>NT-008</v>
       </c>
+      <c r="R121" t="str">
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
@@ -7872,6 +7959,9 @@
       <c r="Q122" t="str">
         <v>NT-005</v>
       </c>
+      <c r="R122" t="str">
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
@@ -8093,6 +8183,9 @@
       <c r="Q126" t="str">
         <v>NT-006</v>
       </c>
+      <c r="R126" t="str">
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
@@ -8762,6 +8855,9 @@
       <c r="Q138" t="str">
         <v>NT-008</v>
       </c>
+      <c r="R138" t="str">
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
@@ -8835,8 +8931,8 @@
       <c r="E140">
         <v>13</v>
       </c>
-      <c r="F140" t="str">
-        <v/>
+      <c r="F140">
+        <v>0</v>
       </c>
       <c r="G140">
         <v>20</v>
@@ -8870,6 +8966,9 @@
       </c>
       <c r="Q140" t="str">
         <v>NT-011</v>
+      </c>
+      <c r="R140" t="str">
+        <v/>
       </c>
     </row>
     <row r="141">
@@ -9540,6 +9639,9 @@
       <c r="Q152" t="str">
         <v>NT-012</v>
       </c>
+      <c r="R152" t="str">
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -9649,6 +9751,9 @@
       <c r="Q154" t="str">
         <v>NT-012</v>
       </c>
+      <c r="R154" t="str">
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -9926,6 +10031,9 @@
       <c r="Q159" t="str">
         <v>NT-005</v>
       </c>
+      <c r="R159" t="str">
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
@@ -9979,6 +10087,9 @@
       <c r="Q160" t="str">
         <v>NT-013</v>
       </c>
+      <c r="R160" t="str">
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
@@ -10032,6 +10143,9 @@
       <c r="Q161" t="str">
         <v>NT-014</v>
       </c>
+      <c r="R161" t="str">
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
@@ -10141,6 +10255,9 @@
       <c r="Q163" t="str">
         <v>NT-011</v>
       </c>
+      <c r="R163" t="str">
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
@@ -10306,6 +10423,9 @@
       <c r="Q166" t="str">
         <v>NT-005</v>
       </c>
+      <c r="R166" t="str">
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
@@ -10359,6 +10479,9 @@
       <c r="Q167" t="str">
         <v>NT-011</v>
       </c>
+      <c r="R167" t="str">
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
@@ -10412,6 +10535,9 @@
       <c r="Q168" t="str">
         <v>NT-011</v>
       </c>
+      <c r="R168" t="str">
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
@@ -10533,10 +10659,10 @@
         <v/>
       </c>
       <c r="C171" t="str">
-        <v>Economia De Lo Publico I</v>
+        <v>Economia De Lo Público I</v>
       </c>
       <c r="D171" t="str">
-        <v>Economia De Lo Publico I</v>
+        <v>Economia De Lo Público I</v>
       </c>
       <c r="E171">
         <v>3</v>
@@ -10689,6 +10815,9 @@
       <c r="Q173" t="str">
         <v>NT-011</v>
       </c>
+      <c r="R173" t="str">
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
@@ -10742,6 +10871,9 @@
       <c r="Q174" t="str">
         <v>NT-005</v>
       </c>
+      <c r="R174" t="str">
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
@@ -11131,6 +11263,9 @@
       <c r="Q181" t="str">
         <v>NT-012</v>
       </c>
+      <c r="R181" t="str">
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
@@ -11184,6 +11319,9 @@
       <c r="Q182" t="str">
         <v>NT-012</v>
       </c>
+      <c r="R182" t="str">
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
@@ -11249,10 +11387,10 @@
         <v/>
       </c>
       <c r="C184" t="str">
-        <v>Economia De Lo Publico II</v>
+        <v>Economia De Lo Público II</v>
       </c>
       <c r="D184" t="str">
-        <v>Economia De Lo Publico II</v>
+        <v>Economia De Lo Público II</v>
       </c>
       <c r="E184">
         <v>3</v>
@@ -11349,6 +11487,9 @@
       <c r="Q185" t="str">
         <v>NT-011</v>
       </c>
+      <c r="R185" t="str">
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
@@ -11682,6 +11823,9 @@
       <c r="Q191" t="str">
         <v>NT-011</v>
       </c>
+      <c r="R191" t="str">
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
@@ -11735,6 +11879,9 @@
       <c r="Q192" t="str">
         <v>NT-014</v>
       </c>
+      <c r="R192" t="str">
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
@@ -11844,6 +11991,9 @@
       <c r="Q194" t="str">
         <v>NT-018</v>
       </c>
+      <c r="R194" t="str">
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
@@ -11953,6 +12103,9 @@
       <c r="Q196" t="str">
         <v>NT-018</v>
       </c>
+      <c r="R196" t="str">
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
@@ -11962,10 +12115,10 @@
         <v/>
       </c>
       <c r="C197" t="str">
-        <v>Gobierno Y Politica Publica</v>
+        <v>Gobierno Y Politica Pública</v>
       </c>
       <c r="D197" t="str">
-        <v>Gobierno Y Politica Publica</v>
+        <v>Gobierno Y Politica Pública</v>
       </c>
       <c r="E197">
         <v>3</v>
@@ -12005,6 +12158,9 @@
       </c>
       <c r="Q197" t="str">
         <v>NT-014</v>
+      </c>
+      <c r="R197" t="str">
+        <v/>
       </c>
     </row>
     <row r="198">
@@ -12059,6 +12215,9 @@
       <c r="Q198" t="str">
         <v>NT-018</v>
       </c>
+      <c r="R198" t="str">
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
@@ -12280,6 +12439,9 @@
       <c r="Q202" t="str">
         <v>NT-017</v>
       </c>
+      <c r="R202" t="str">
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
@@ -12345,10 +12507,10 @@
         <v/>
       </c>
       <c r="C204" t="str">
-        <v>Problemática Publica Colombiana</v>
+        <v>Problemática Pública Colombiana</v>
       </c>
       <c r="D204" t="str">
-        <v>Problemática Publica Colombiana</v>
+        <v>Problemática Pública Colombiana</v>
       </c>
       <c r="E204">
         <v>2</v>
@@ -12445,6 +12607,9 @@
       <c r="Q205" t="str">
         <v>NT-018</v>
       </c>
+      <c r="R205" t="str">
+        <v/>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
@@ -12778,6 +12943,9 @@
       <c r="Q211" t="str">
         <v>NT-018</v>
       </c>
+      <c r="R211" t="str">
+        <v/>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
@@ -13111,6 +13279,9 @@
       <c r="Q217" t="str">
         <v>NT-018</v>
       </c>
+      <c r="R217" t="str">
+        <v/>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
@@ -13184,8 +13355,8 @@
       <c r="E219">
         <v>13</v>
       </c>
-      <c r="F219" t="str">
-        <v/>
+      <c r="F219">
+        <v>0</v>
       </c>
       <c r="G219">
         <v>144</v>
@@ -13219,6 +13390,9 @@
       </c>
       <c r="Q219" t="str">
         <v>NT-011</v>
+      </c>
+      <c r="R219" t="str">
+        <v/>
       </c>
     </row>
     <row r="220">
@@ -13273,6 +13447,9 @@
       <c r="Q220" t="str">
         <v>NT-011</v>
       </c>
+      <c r="R220" t="str">
+        <v/>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
@@ -13324,7 +13501,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q221" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="R221" t="str">
         <v>AF-17</v>
@@ -13380,7 +13557,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q222" t="str">
-        <v/>
+        <v>NT-035</v>
       </c>
       <c r="R222" t="str">
         <v>AF-17</v>
@@ -14166,6 +14343,9 @@
       <c r="Q236" t="str">
         <v>NT-020</v>
       </c>
+      <c r="R236" t="str">
+        <v/>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
@@ -15399,6 +15579,9 @@
       <c r="Q258" t="str">
         <v>NT-006</v>
       </c>
+      <c r="R258" t="str">
+        <v/>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
@@ -15900,6 +16083,9 @@
       <c r="Q267" t="str">
         <v>NT-006</v>
       </c>
+      <c r="R267" t="str">
+        <v/>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
@@ -16021,10 +16207,10 @@
         <v/>
       </c>
       <c r="C270" t="str">
-        <v>Economía Publica y Política Fiscal</v>
+        <v>Economía Pública y Política Fiscal</v>
       </c>
       <c r="D270" t="str">
-        <v>Economía Publica y Política Fiscal</v>
+        <v>Economía Pública y Política Fiscal</v>
       </c>
       <c r="E270">
         <v>3</v>
@@ -16693,10 +16879,10 @@
         <v/>
       </c>
       <c r="C282" t="str">
-        <v>Teorías y Problemas de la Administración Publica</v>
+        <v>Teorías y Problemas de la Administración Pública</v>
       </c>
       <c r="D282" t="str">
-        <v>Teorías y Problemas de la Administración Publica</v>
+        <v>Teorías y Problemas de la Administración Pública</v>
       </c>
       <c r="E282">
         <v>3</v>
@@ -24881,8 +25067,8 @@
       <c r="E428">
         <v>13</v>
       </c>
-      <c r="F428" t="str">
-        <v/>
+      <c r="F428">
+        <v>0</v>
       </c>
       <c r="G428">
         <v>20</v>
@@ -24916,6 +25102,9 @@
       </c>
       <c r="Q428" t="str">
         <v>NT-011</v>
+      </c>
+      <c r="R428" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -42598,7 +42787,7 @@
         <v>PRO-003</v>
       </c>
       <c r="C53" t="str">
-        <v>Gobierno Y Politica Publica</v>
+        <v>Gobierno Y Politica Pública</v>
       </c>
       <c r="D53" t="str">
         <v>Problemática Del  Estado Y Del Poder</v>
@@ -43007,1531 +43196,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G66"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>codigo_actual</v>
-      </c>
-      <c r="B1" t="str">
-        <v>asignatura</v>
-      </c>
-      <c r="C1" t="str">
-        <v>area_anterior</v>
-      </c>
-      <c r="D1" t="str">
-        <v>area_importar</v>
-      </c>
-      <c r="E1" t="str">
-        <v>codigo_nt</v>
-      </c>
-      <c r="F1" t="str">
-        <v>codigo_af</v>
-      </c>
-      <c r="G1" t="str">
-        <v>planes_fuente</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>ASIG-00002</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Construcción Del Territorio</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Desarrollo Y Gestión Territorial</v>
-      </c>
-      <c r="E2" t="str">
-        <v>NT-007</v>
-      </c>
-      <c r="F2" t="str">
-        <v>AF-05</v>
-      </c>
-      <c r="G2" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ASIG-00003</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Fundamentos De Economía Pública</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Finanzas Públicas</v>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v>AF-04</v>
-      </c>
-      <c r="G3" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>ASIG-00004</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Fundamentos De Economía Pública</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Finanzas Públicas</v>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v>AF-04</v>
-      </c>
-      <c r="G4" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>ASIG-00005</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Fundamentos Sociológicos</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E5" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F5" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G5" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>ASIG-00006</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Historia de la administración pública</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E6" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F6" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G6" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>ASIG-00007</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Historia de la administración pública</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E7" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F7" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G7" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>ASIG-00008</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Historia Del Pensamiento Político</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E8" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F8" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G8" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>ASIG-00013</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Matemáticas I</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E9" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F9" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G9" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>ASIG-00014</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Matemáticas Lúdicas</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E10" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F10" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G10" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>ASIG-00015</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Matemáticas Lúdicas</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E11" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F11" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G11" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>ASIG-00021</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Sistemas Informáticos</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E12" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F12" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G12" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>ASIG-00022</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Sistemas Informáticos</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E13" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F13" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G13" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>ASIG-00023</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Taller de Lectoescritura</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D14" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E14" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F14" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G14" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>ASIG-00024</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Taller de Lectoescritura</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D15" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E15" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F15" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G15" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>ASIG-00026</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Derecho Constitucional</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D16" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E16" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F16" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G16" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>ASIG-00027</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Derecho Constitucional</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D17" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E17" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F17" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G17" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>ASIG-00030</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Electiva I</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D18" t="str">
-        <v>Electivas Generales</v>
-      </c>
-      <c r="E18" t="str">
-        <v>NT-009</v>
-      </c>
-      <c r="F18" t="str">
-        <v>AF-12</v>
-      </c>
-      <c r="G18" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>ASIG-00031</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Fundamentos Sociológicos</v>
-      </c>
-      <c r="C19" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D19" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E19" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F19" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G19" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>ASIG-00035</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Macroeconomía y Política Económica</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Finanzas Públicas</v>
-      </c>
-      <c r="E20" t="str">
-        <v/>
-      </c>
-      <c r="F20" t="str">
-        <v>AF-04</v>
-      </c>
-      <c r="G20" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>ASIG-00036</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Macroeconomía y Política Económica</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Finanzas Públicas</v>
-      </c>
-      <c r="E21" t="str">
-        <v/>
-      </c>
-      <c r="F21" t="str">
-        <v>AF-04</v>
-      </c>
-      <c r="G21" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>ASIG-00038</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Matemáticas I</v>
-      </c>
-      <c r="C22" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E22" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F22" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G22" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>ASIG-00041</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Organización Estatal Colombiana</v>
-      </c>
-      <c r="C23" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E23" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F23" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G23" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>ASIG-00042</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Organización Estatal Colombiana</v>
-      </c>
-      <c r="C24" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D24" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E24" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F24" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G24" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>ASIG-00058</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Finanzas y análisis financiero público</v>
-      </c>
-      <c r="C25" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Finanzas Públicas</v>
-      </c>
-      <c r="E25" t="str">
-        <v/>
-      </c>
-      <c r="F25" t="str">
-        <v>AF-04</v>
-      </c>
-      <c r="G25" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>ASIG-00059</v>
-      </c>
-      <c r="B26" t="str">
-        <v>Teorías del Estado y regímenes políticos</v>
-      </c>
-      <c r="C26" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E26" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F26" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G26" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>ASIG-00060</v>
-      </c>
-      <c r="B27" t="str">
-        <v>Demografía</v>
-      </c>
-      <c r="C27" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E27" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F27" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G27" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>ASIG-00061</v>
-      </c>
-      <c r="B28" t="str">
-        <v>Pensamientos y teorías de la administración pública</v>
-      </c>
-      <c r="C28" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D28" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E28" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F28" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G28" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>ASIG-00062</v>
-      </c>
-      <c r="B29" t="str">
-        <v>Matemáticas II</v>
-      </c>
-      <c r="C29" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D29" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E29" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F29" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G29" t="str">
-        <v>AP_35</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>ASIG-00063</v>
-      </c>
-      <c r="B30" t="str">
-        <v>Finanzas y análisis financiero público</v>
-      </c>
-      <c r="C30" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D30" t="str">
-        <v>Finanzas Públicas</v>
-      </c>
-      <c r="E30" t="str">
-        <v/>
-      </c>
-      <c r="F30" t="str">
-        <v>AF-04</v>
-      </c>
-      <c r="G30" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>ASIG-00066</v>
-      </c>
-      <c r="B31" t="str">
-        <v>Pensamientos y teorías de la administración pública</v>
-      </c>
-      <c r="C31" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
-      </c>
-      <c r="D31" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E31" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F31" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G31" t="str">
-        <v>AP_36</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>ASIG-00146</v>
-      </c>
-      <c r="B32" t="str">
-        <v>Fundamentos de economía pública</v>
-      </c>
-      <c r="C32" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D32" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="E32" t="str">
-        <v>NT-006</v>
-      </c>
-      <c r="F32" t="str">
-        <v>AF-03</v>
-      </c>
-      <c r="G32" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>ASIG-00147</v>
-      </c>
-      <c r="B33" t="str">
-        <v>Fundamentos del Estado y el poder</v>
-      </c>
-      <c r="C33" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D33" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E33" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F33" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G33" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>ASIG-00148</v>
-      </c>
-      <c r="B34" t="str">
-        <v>Fundamentos sociológicos</v>
-      </c>
-      <c r="C34" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D34" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E34" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F34" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G34" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>ASIG-00149</v>
-      </c>
-      <c r="B35" t="str">
-        <v>Geografía física y ambiental</v>
-      </c>
-      <c r="C35" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D35" t="str">
-        <v>Desarrollo Y Gestión Territorial</v>
-      </c>
-      <c r="E35" t="str">
-        <v>NT-007</v>
-      </c>
-      <c r="F35" t="str">
-        <v>AF-05</v>
-      </c>
-      <c r="G35" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>ASIG-00150</v>
-      </c>
-      <c r="B36" t="str">
-        <v>Historia de la administración pública</v>
-      </c>
-      <c r="C36" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D36" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E36" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F36" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G36" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>ASIG-00152</v>
-      </c>
-      <c r="B37" t="str">
-        <v>Geografía económica y social</v>
-      </c>
-      <c r="C37" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D37" t="str">
-        <v>Desarrollo Y Gestión Territorial</v>
-      </c>
-      <c r="E37" t="str">
-        <v>NT-007</v>
-      </c>
-      <c r="F37" t="str">
-        <v>AF-05</v>
-      </c>
-      <c r="G37" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>ASIG-00154</v>
-      </c>
-      <c r="B38" t="str">
-        <v>Micro y macroeconomía</v>
-      </c>
-      <c r="C38" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D38" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="E38" t="str">
-        <v>NT-006</v>
-      </c>
-      <c r="F38" t="str">
-        <v>AF-03</v>
-      </c>
-      <c r="G38" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>ASIG-00155</v>
-      </c>
-      <c r="B39" t="str">
-        <v>Pensamientos y teorías de la administración pública</v>
-      </c>
-      <c r="C39" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D39" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E39" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F39" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G39" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>ASIG-00156</v>
-      </c>
-      <c r="B40" t="str">
-        <v>Regímenes y sistemas políticos</v>
-      </c>
-      <c r="C40" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D40" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E40" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F40" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G40" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>ASIG-00157</v>
-      </c>
-      <c r="B41" t="str">
-        <v>Socialización y cultura</v>
-      </c>
-      <c r="C41" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D41" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E41" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F41" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G41" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>ASIG-00163</v>
-      </c>
-      <c r="B42" t="str">
-        <v>Electiva I</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="D42" t="str">
-        <v>Formación General</v>
-      </c>
-      <c r="E42" t="str">
-        <v>NT-011</v>
-      </c>
-      <c r="F42" t="str">
-        <v>AF-18</v>
-      </c>
-      <c r="G42" t="str">
-        <v>APT_52</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>ASIG-00176</v>
-      </c>
-      <c r="B43" t="str">
-        <v>Teorías de las organizaciones públicas</v>
-      </c>
-      <c r="C43" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D43" t="str">
-        <v>Organizaciones Públicas</v>
-      </c>
-      <c r="E43" t="str">
-        <v>NT-017</v>
-      </c>
-      <c r="F43" t="str">
-        <v>AF-02</v>
-      </c>
-      <c r="G43" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v>ASIG-00177</v>
-      </c>
-      <c r="B44" t="str">
-        <v>Derecho constitucional</v>
-      </c>
-      <c r="C44" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D44" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E44" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F44" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G44" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <v>ASIG-00178</v>
-      </c>
-      <c r="B45" t="str">
-        <v>Actores sociales y diferencia identitaria</v>
-      </c>
-      <c r="C45" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D45" t="str">
-        <v>Estado, Gobierno y Sociedad</v>
-      </c>
-      <c r="E45" t="str">
-        <v>NT-013</v>
-      </c>
-      <c r="F45" t="str">
-        <v>AF-10</v>
-      </c>
-      <c r="G45" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>ASIG-00179</v>
-      </c>
-      <c r="B46" t="str">
-        <v>Finanzas y análisis financiero público</v>
-      </c>
-      <c r="C46" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D46" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="E46" t="str">
-        <v>NT-006</v>
-      </c>
-      <c r="F46" t="str">
-        <v>AF-03</v>
-      </c>
-      <c r="G46" t="str">
-        <v>APT_53</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>ASIG-00220</v>
-      </c>
-      <c r="B47" t="str">
-        <v>Seminario Electivo I</v>
-      </c>
-      <c r="C47" t="str">
-        <v>Formación General</v>
-      </c>
-      <c r="D47" t="str">
-        <v>Opción de grado</v>
-      </c>
-      <c r="E47" t="str">
-        <v/>
-      </c>
-      <c r="F47" t="str">
-        <v>AF-17</v>
-      </c>
-      <c r="G47" t="str">
-        <v>APT_52</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>ASIG-00221</v>
-      </c>
-      <c r="B48" t="str">
-        <v>Seminario Electivo II</v>
-      </c>
-      <c r="C48" t="str">
-        <v>Formación General</v>
-      </c>
-      <c r="D48" t="str">
-        <v>Opción de grado</v>
-      </c>
-      <c r="E48" t="str">
-        <v/>
-      </c>
-      <c r="F48" t="str">
-        <v>AF-17</v>
-      </c>
-      <c r="G48" t="str">
-        <v>APT_52</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>ASIG-00224</v>
-      </c>
-      <c r="B49" t="str">
-        <v>Fundamentos Administración Pública.</v>
-      </c>
-      <c r="C49" t="str">
-        <v>Teoría Económica e Historia</v>
-      </c>
-      <c r="D49" t="str">
-        <v>Formación integral Y de contexto</v>
-      </c>
-      <c r="E49" t="str">
-        <v>NT-021</v>
-      </c>
-      <c r="F49" t="str">
-        <v>AF-16</v>
-      </c>
-      <c r="G49" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <v>ASIG-00231</v>
-      </c>
-      <c r="B50" t="str">
-        <v>Fundamentos de Contabilidad</v>
-      </c>
-      <c r="C50" t="str">
-        <v>Formación integral Y de contexto</v>
-      </c>
-      <c r="D50" t="str">
-        <v>Teoría Económica e Historia</v>
-      </c>
-      <c r="E50" t="str">
-        <v>NT-022</v>
-      </c>
-      <c r="F50" t="str">
-        <v>AF-15</v>
-      </c>
-      <c r="G50" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>ASIG-00249</v>
-      </c>
-      <c r="B51" t="str">
-        <v>Bienes Públicos, Servicios Públicos y Regulación</v>
-      </c>
-      <c r="C51" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D51" t="str">
-        <v>Teoría Económica e Historia</v>
-      </c>
-      <c r="E51" t="str">
-        <v>NT-022</v>
-      </c>
-      <c r="F51" t="str">
-        <v>AF-15</v>
-      </c>
-      <c r="G51" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="52" xml:space="preserve">
-      <c r="A52" t="str">
-        <v>ASIG-00250</v>
-      </c>
-      <c r="B52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Contabilidad
-Gubernamental</v>
-      </c>
-      <c r="C52" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D52" t="str">
-        <v>Teoría Económica e Historia</v>
-      </c>
-      <c r="E52" t="str">
-        <v>NT-022</v>
-      </c>
-      <c r="F52" t="str">
-        <v>AF-15</v>
-      </c>
-      <c r="G52" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>ASIG-00251</v>
-      </c>
-      <c r="B53" t="str">
-        <v>Curso electivo 2</v>
-      </c>
-      <c r="C53" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D53" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E53" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F53" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G53" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>ASIG-00252</v>
-      </c>
-      <c r="B54" t="str">
-        <v>Economía Política</v>
-      </c>
-      <c r="C54" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D54" t="str">
-        <v>Teoría Económica e Historia</v>
-      </c>
-      <c r="E54" t="str">
-        <v>NT-022</v>
-      </c>
-      <c r="F54" t="str">
-        <v>AF-15</v>
-      </c>
-      <c r="G54" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>ASIG-00253</v>
-      </c>
-      <c r="B55" t="str">
-        <v>Fundamentos Economía Pública</v>
-      </c>
-      <c r="C55" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D55" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E55" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F55" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G55" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="56" xml:space="preserve">
-      <c r="A56" t="str">
-        <v>ASIG-00254</v>
-      </c>
-      <c r="B56" t="str" xml:space="preserve">
-        <v xml:space="preserve">Déficit fiscal y
-deuda pública</v>
-      </c>
-      <c r="C56" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D56" t="str">
-        <v>Teoría Económica e Historia</v>
-      </c>
-      <c r="E56" t="str">
-        <v>NT-022</v>
-      </c>
-      <c r="F56" t="str">
-        <v>AF-15</v>
-      </c>
-      <c r="G56" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>ASIG-00255</v>
-      </c>
-      <c r="B57" t="str">
-        <v>Desarrollo Económico y Regional</v>
-      </c>
-      <c r="C57" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D57" t="str">
-        <v>Formación integral Y de contexto</v>
-      </c>
-      <c r="E57" t="str">
-        <v>NT-021</v>
-      </c>
-      <c r="F57" t="str">
-        <v>AF-16</v>
-      </c>
-      <c r="G57" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>ASIG-00256</v>
-      </c>
-      <c r="B58" t="str">
-        <v>Economía Ambiental y Desarrollo Sostenible</v>
-      </c>
-      <c r="C58" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D58" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E58" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F58" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G58" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>ASIG-00258</v>
-      </c>
-      <c r="B59" t="str">
-        <v>Gestión y Gerencia Pública.</v>
-      </c>
-      <c r="C59" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D59" t="str">
-        <v>Formación integral Y de contexto</v>
-      </c>
-      <c r="E59" t="str">
-        <v>NT-021</v>
-      </c>
-      <c r="F59" t="str">
-        <v>AF-16</v>
-      </c>
-      <c r="G59" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>ASIG-00259</v>
-      </c>
-      <c r="B60" t="str">
-        <v>Ingresos Públicos (y Tributación) (Nacional, territorial</v>
-      </c>
-      <c r="C60" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D60" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E60" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F60" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G60" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>ASIG-00260</v>
-      </c>
-      <c r="B61" t="str">
-        <v>Contratación pública</v>
-      </c>
-      <c r="C61" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D61" t="str">
-        <v>Formación integral Y de contexto</v>
-      </c>
-      <c r="E61" t="str">
-        <v>NT-021</v>
-      </c>
-      <c r="F61" t="str">
-        <v>AF-16</v>
-      </c>
-      <c r="G61" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>ASIG-00261</v>
-      </c>
-      <c r="B62" t="str">
-        <v>Curso Electivo 3</v>
-      </c>
-      <c r="C62" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D62" t="str">
-        <v>Formación integral Y de contexto</v>
-      </c>
-      <c r="E62" t="str">
-        <v>NT-021</v>
-      </c>
-      <c r="F62" t="str">
-        <v>AF-16</v>
-      </c>
-      <c r="G62" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>ASIG-00262</v>
-      </c>
-      <c r="B63" t="str">
-        <v>Formulación y Evaluación Económica y Social de Proyectos</v>
-      </c>
-      <c r="C63" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D63" t="str">
-        <v>Teoría Económica e Historia</v>
-      </c>
-      <c r="E63" t="str">
-        <v>NT-022</v>
-      </c>
-      <c r="F63" t="str">
-        <v>AF-15</v>
-      </c>
-      <c r="G63" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>ASIG-00263</v>
-      </c>
-      <c r="B64" t="str">
-        <v>Gestión Financiera pública.</v>
-      </c>
-      <c r="C64" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D64" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E64" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F64" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G64" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="str">
-        <v>ASIG-00264</v>
-      </c>
-      <c r="B65" t="str">
-        <v>Política Económica y Social</v>
-      </c>
-      <c r="C65" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D65" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E65" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F65" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G65" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="str">
-        <v>ASIG-00265</v>
-      </c>
-      <c r="B66" t="str">
-        <v>Presupuesto Público (Nacional, Territorial.</v>
-      </c>
-      <c r="C66" t="str">
-        <v>Economía Pública</v>
-      </c>
-      <c r="D66" t="str">
-        <v>Teoría Económica e Historia</v>
-      </c>
-      <c r="E66" t="str">
-        <v>NT-022</v>
-      </c>
-      <c r="F66" t="str">
-        <v>AF-15</v>
-      </c>
-      <c r="G66" t="str">
-        <v>EP_37D | EP_37N</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Areas conciliadas y Excel final, consulta de periodos sin escritura, parche de consola y envio a revision verificado
- generar-catalogo: una decision de area que ya se cumple conserva el nucleo actual (18 cambios exactos, no 26); Excel regenerado.
- GET /periodos-academicos ya no siembra un periodo; prueba nueva.
- ProgramacionAcademicaModule: no consulta jefatura con la concertacion encendida.
- INTEGRACION-claude.md s30.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/esap/programacion/resultados/2026-1/catalogo-importable-2026-1.xlsx
+++ b/esap/programacion/resultados/2026-1/catalogo-importable-2026-1.xlsx
@@ -1833,7 +1833,7 @@
         <v>presencial_noche</v>
       </c>
       <c r="J13" t="str">
-        <v>Cuantitativa</v>
+        <v>Fundamentación Cuantitativa</v>
       </c>
       <c r="K13" t="str">
         <v>PRO-002</v>
@@ -1854,7 +1854,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q13" t="str">
-        <v>NT-020</v>
+        <v>NT-004</v>
       </c>
       <c r="R13" t="str">
         <v>AF-07</v>
@@ -3233,7 +3233,7 @@
         <v>presencial_dia</v>
       </c>
       <c r="J38" t="str">
-        <v>Cuantitativa</v>
+        <v>Fundamentación Cuantitativa</v>
       </c>
       <c r="K38" t="str">
         <v>PRO-001</v>
@@ -3254,7 +3254,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q38" t="str">
-        <v>NT-020</v>
+        <v>NT-004</v>
       </c>
       <c r="R38" t="str">
         <v>AF-07</v>
@@ -3345,7 +3345,7 @@
         <v>presencial_dia</v>
       </c>
       <c r="J40" t="str">
-        <v>Cuantitativa</v>
+        <v>Fundamentación Cuantitativa</v>
       </c>
       <c r="K40" t="str">
         <v>PRO-001</v>
@@ -3366,7 +3366,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q40" t="str">
-        <v>NT-020</v>
+        <v>NT-004</v>
       </c>
       <c r="R40" t="str">
         <v>AF-07</v>
@@ -3401,7 +3401,7 @@
         <v>presencial_noche</v>
       </c>
       <c r="J41" t="str">
-        <v>Cuantitativa</v>
+        <v>Fundamentación Cuantitativa</v>
       </c>
       <c r="K41" t="str">
         <v>PRO-002</v>
@@ -3422,7 +3422,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q41" t="str">
-        <v>NT-020</v>
+        <v>NT-004</v>
       </c>
       <c r="R41" t="str">
         <v>AF-07</v>
@@ -3961,7 +3961,7 @@
         <v>presencial_dia</v>
       </c>
       <c r="J51" t="str">
-        <v>Cuantitativa</v>
+        <v>Fundamentación Cuantitativa</v>
       </c>
       <c r="K51" t="str">
         <v>PRO-001</v>
@@ -3982,7 +3982,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q51" t="str">
-        <v>NT-020</v>
+        <v>NT-004</v>
       </c>
       <c r="R51" t="str">
         <v>AF-07</v>
@@ -4017,7 +4017,7 @@
         <v>presencial_noche</v>
       </c>
       <c r="J52" t="str">
-        <v>Cuantitativa</v>
+        <v>Fundamentación Cuantitativa</v>
       </c>
       <c r="K52" t="str">
         <v>PRO-002</v>
@@ -4038,7 +4038,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q52" t="str">
-        <v>NT-020</v>
+        <v>NT-004</v>
       </c>
       <c r="R52" t="str">
         <v>AF-07</v>
@@ -5081,7 +5081,7 @@
         <v>presencial_dia</v>
       </c>
       <c r="J71" t="str">
-        <v>Cuantitativa</v>
+        <v>Fundamentación Cuantitativa</v>
       </c>
       <c r="K71" t="str">
         <v>PRO-001</v>
@@ -5102,7 +5102,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q71" t="str">
-        <v>NT-020</v>
+        <v>NT-004</v>
       </c>
       <c r="R71" t="str">
         <v>AF-07</v>
@@ -5137,7 +5137,7 @@
         <v>presencial_noche</v>
       </c>
       <c r="J72" t="str">
-        <v>Cuantitativa</v>
+        <v>Fundamentación Cuantitativa</v>
       </c>
       <c r="K72" t="str">
         <v>PRO-002</v>
@@ -5158,7 +5158,7 @@
         <v>TRUE</v>
       </c>
       <c r="Q72" t="str">
-        <v>NT-020</v>
+        <v>NT-004</v>
       </c>
       <c r="R72" t="str">
         <v>AF-07</v>
@@ -42807,7 +42807,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -42857,13 +42857,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ASIG-00012</v>
+        <v>ASIG-00013</v>
       </c>
       <c r="B3" t="str">
-        <v>Matemática I</v>
+        <v>Matemáticas I</v>
       </c>
       <c r="C3" t="str">
-        <v>Fundamentación Cuantitativa</v>
+        <v>Complementaria</v>
       </c>
       <c r="D3" t="str">
         <v>Cuantitativa</v>
@@ -42875,15 +42875,15 @@
         <v>AF-07</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>AP_35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ASIG-00013</v>
+        <v>ASIG-00014</v>
       </c>
       <c r="B4" t="str">
-        <v>Matemáticas I</v>
+        <v>Matemáticas Lúdicas</v>
       </c>
       <c r="C4" t="str">
         <v>Complementaria</v>
@@ -42903,7 +42903,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>ASIG-00014</v>
+        <v>ASIG-00015</v>
       </c>
       <c r="B5" t="str">
         <v>Matemáticas Lúdicas</v>
@@ -42921,15 +42921,15 @@
         <v>AF-07</v>
       </c>
       <c r="G5" t="str">
-        <v>AP_35</v>
+        <v>AP_36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>ASIG-00015</v>
+        <v>ASIG-00038</v>
       </c>
       <c r="B6" t="str">
-        <v>Matemáticas Lúdicas</v>
+        <v>Matemáticas I</v>
       </c>
       <c r="C6" t="str">
         <v>Complementaria</v>
@@ -42949,13 +42949,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>ASIG-00037</v>
+        <v>ASIG-00062</v>
       </c>
       <c r="B7" t="str">
-        <v>Matemáticas I</v>
+        <v>Matemáticas II</v>
       </c>
       <c r="C7" t="str">
-        <v>Fundamentación Cuantitativa</v>
+        <v>Complementaria</v>
       </c>
       <c r="D7" t="str">
         <v>Cuantitativa</v>
@@ -42967,64 +42967,64 @@
         <v>AF-07</v>
       </c>
       <c r="G7" t="str">
-        <v>AP_33</v>
+        <v>AP_35</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>ASIG-00038</v>
+        <v>ASIG-00064</v>
       </c>
       <c r="B8" t="str">
-        <v>Matemáticas I</v>
+        <v>Historia del pensamiento político (AP_noche) Nuevo Plan de Estudios</v>
       </c>
       <c r="C8" t="str">
-        <v>Complementaria</v>
+        <v>Nuevo Plan de Estudios AP</v>
       </c>
       <c r="D8" t="str">
-        <v>Cuantitativa</v>
+        <v>Estado Y Poder</v>
       </c>
       <c r="E8" t="str">
-        <v>NT-020</v>
+        <v>NT-002</v>
       </c>
       <c r="F8" t="str">
-        <v>AF-07</v>
+        <v>AF-01</v>
       </c>
       <c r="G8" t="str">
-        <v>AP_36</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>ASIG-00039</v>
+        <v>ASIG-00065</v>
       </c>
       <c r="B9" t="str">
-        <v>Matemáticas II</v>
+        <v>Electiva I (AP_noche) Nuevo Plan de Estudios</v>
       </c>
       <c r="C9" t="str">
-        <v>Fundamentación Cuantitativa</v>
+        <v>Nuevo Plan de Estudios AP</v>
       </c>
       <c r="D9" t="str">
-        <v>Cuantitativa</v>
+        <v>Electivas Generales</v>
       </c>
       <c r="E9" t="str">
-        <v>NT-020</v>
+        <v>NT-009</v>
       </c>
       <c r="F9" t="str">
-        <v>AF-07</v>
+        <v>AF-12</v>
       </c>
       <c r="G9" t="str">
-        <v>AP_33</v>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>ASIG-00040</v>
+        <v>ASIG-00067</v>
       </c>
       <c r="B10" t="str">
-        <v>Matemáticas II</v>
+        <v>Matemáticas II (AP_noche) Nuevo Plan de Estudios</v>
       </c>
       <c r="C10" t="str">
-        <v>Fundamentación Cuantitativa</v>
+        <v>Nuevo Plan de Estudios AP</v>
       </c>
       <c r="D10" t="str">
         <v>Cuantitativa</v>
@@ -43036,18 +43036,18 @@
         <v>AF-07</v>
       </c>
       <c r="G10" t="str">
-        <v>AP_34</v>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>ASIG-00050</v>
+        <v>ASIG-00151</v>
       </c>
       <c r="B11" t="str">
-        <v>Estadística I</v>
+        <v>Matemática I</v>
       </c>
       <c r="C11" t="str">
-        <v>Fundamentación Cuantitativa</v>
+        <v>Nuevo Plan de Estudios APT</v>
       </c>
       <c r="D11" t="str">
         <v>Cuantitativa</v>
@@ -43059,18 +43059,18 @@
         <v>AF-07</v>
       </c>
       <c r="G11" t="str">
-        <v>AP_33</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>ASIG-00051</v>
+        <v>ASIG-00153</v>
       </c>
       <c r="B12" t="str">
-        <v>Estadística I</v>
+        <v>Matemáticas II</v>
       </c>
       <c r="C12" t="str">
-        <v>Fundamentación Cuantitativa</v>
+        <v>Nuevo Plan de Estudios APT</v>
       </c>
       <c r="D12" t="str">
         <v>Cuantitativa</v>
@@ -43082,18 +43082,18 @@
         <v>AF-07</v>
       </c>
       <c r="G12" t="str">
-        <v>AP_34</v>
+        <v>APT_52 | APT_53</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>ASIG-00062</v>
+        <v>ASIG-00162</v>
       </c>
       <c r="B13" t="str">
-        <v>Matemáticas II</v>
+        <v>Matemática I</v>
       </c>
       <c r="C13" t="str">
-        <v>Complementaria</v>
+        <v>Formación General</v>
       </c>
       <c r="D13" t="str">
         <v>Cuantitativa</v>
@@ -43105,27 +43105,27 @@
         <v>AF-07</v>
       </c>
       <c r="G13" t="str">
-        <v>AP_35</v>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>ASIG-00064</v>
+        <v>ASIG-00167</v>
       </c>
       <c r="B14" t="str">
-        <v>Historia del pensamiento político (AP_noche) Nuevo Plan de Estudios</v>
+        <v>Matemática II</v>
       </c>
       <c r="C14" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
+        <v>Formación General</v>
       </c>
       <c r="D14" t="str">
-        <v>Estado Y Poder</v>
+        <v>Cuantitativa</v>
       </c>
       <c r="E14" t="str">
-        <v>NT-002</v>
+        <v>NT-020</v>
       </c>
       <c r="F14" t="str">
-        <v>AF-01</v>
+        <v>AF-07</v>
       </c>
       <c r="G14" t="str">
         <v/>
@@ -43133,36 +43133,36 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>ASIG-00065</v>
+        <v>ASIG-00172</v>
       </c>
       <c r="B15" t="str">
-        <v>Electiva I (AP_noche) Nuevo Plan de Estudios</v>
+        <v>Estadistica I</v>
       </c>
       <c r="C15" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
+        <v>Formación General</v>
       </c>
       <c r="D15" t="str">
-        <v>Electivas Generales</v>
+        <v>Cuantitativa</v>
       </c>
       <c r="E15" t="str">
-        <v>NT-009</v>
+        <v>NT-020</v>
       </c>
       <c r="F15" t="str">
-        <v>AF-12</v>
+        <v>AF-07</v>
       </c>
       <c r="G15" t="str">
-        <v/>
+        <v>APT_52 | APT_53</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ASIG-00067</v>
+        <v>ASIG-00180</v>
       </c>
       <c r="B16" t="str">
-        <v>Matemáticas II (AP_noche) Nuevo Plan de Estudios</v>
+        <v>Estadística I</v>
       </c>
       <c r="C16" t="str">
-        <v>Nuevo Plan de Estudios AP</v>
+        <v>Nuevo Plan de Estudios APT</v>
       </c>
       <c r="D16" t="str">
         <v>Cuantitativa</v>
@@ -43174,41 +43174,41 @@
         <v>AF-07</v>
       </c>
       <c r="G16" t="str">
-        <v/>
+        <v>APT_52 | APT_53</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ASIG-00070</v>
+        <v>ASIG-00181</v>
       </c>
       <c r="B17" t="str">
-        <v>Estadística II</v>
+        <v>Metodología de investigación</v>
       </c>
       <c r="C17" t="str">
-        <v>Fundamentación Cuantitativa</v>
+        <v>Nuevo Plan de Estudios APT</v>
       </c>
       <c r="D17" t="str">
-        <v>Cuantitativa</v>
+        <v>Complementaria</v>
       </c>
       <c r="E17" t="str">
-        <v>NT-020</v>
+        <v>NT-015</v>
       </c>
       <c r="F17" t="str">
-        <v>AF-07</v>
+        <v>AF-13</v>
       </c>
       <c r="G17" t="str">
-        <v>AP_33</v>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>ASIG-00071</v>
+        <v>ASIG-00184</v>
       </c>
       <c r="B18" t="str">
         <v>Estadística II</v>
       </c>
       <c r="C18" t="str">
-        <v>Fundamentación Cuantitativa</v>
+        <v>Formación General</v>
       </c>
       <c r="D18" t="str">
         <v>Cuantitativa</v>
@@ -43220,18 +43220,18 @@
         <v>AF-07</v>
       </c>
       <c r="G18" t="str">
-        <v>AP_34</v>
+        <v>APT_52 | APT_53</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>ASIG-00151</v>
+        <v>ASIG-00190</v>
       </c>
       <c r="B19" t="str">
-        <v>Matemática I</v>
+        <v>Matematica Financiera</v>
       </c>
       <c r="C19" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
+        <v>Formación General</v>
       </c>
       <c r="D19" t="str">
         <v>Cuantitativa</v>
@@ -43246,193 +43246,9 @@
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>ASIG-00153</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Matemáticas II</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E20" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F20" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G20" t="str">
-        <v>APT_52 | APT_53</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>ASIG-00162</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Matemática I</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Formación General</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E21" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F21" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G21" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>ASIG-00167</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Matemática II</v>
-      </c>
-      <c r="C22" t="str">
-        <v>Formación General</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E22" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F22" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>ASIG-00172</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Estadistica I</v>
-      </c>
-      <c r="C23" t="str">
-        <v>Formación General</v>
-      </c>
-      <c r="D23" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E23" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F23" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G23" t="str">
-        <v>APT_52 | APT_53</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>ASIG-00180</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Estadística I</v>
-      </c>
-      <c r="C24" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D24" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E24" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F24" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G24" t="str">
-        <v>APT_52 | APT_53</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>ASIG-00181</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Metodología de investigación</v>
-      </c>
-      <c r="C25" t="str">
-        <v>Nuevo Plan de Estudios APT</v>
-      </c>
-      <c r="D25" t="str">
-        <v>Complementaria</v>
-      </c>
-      <c r="E25" t="str">
-        <v>NT-015</v>
-      </c>
-      <c r="F25" t="str">
-        <v>AF-13</v>
-      </c>
-      <c r="G25" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>ASIG-00184</v>
-      </c>
-      <c r="B26" t="str">
-        <v>Estadística II</v>
-      </c>
-      <c r="C26" t="str">
-        <v>Formación General</v>
-      </c>
-      <c r="D26" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E26" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F26" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G26" t="str">
-        <v>APT_52 | APT_53</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>ASIG-00190</v>
-      </c>
-      <c r="B27" t="str">
-        <v>Matematica Financiera</v>
-      </c>
-      <c r="C27" t="str">
-        <v>Formación General</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Cuantitativa</v>
-      </c>
-      <c r="E27" t="str">
-        <v>NT-020</v>
-      </c>
-      <c r="F27" t="str">
-        <v>AF-07</v>
-      </c>
-      <c r="G27" t="str">
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>